<commit_message>
Se realizo flujo de caja y plan de costos
Se realizo Flujo de caja y El plan de costos, además se adapto la cantidad de suscripciones.
</commit_message>
<xml_diff>
--- a/Evidencias del Proyecto/Presupuesto proyecto IncluShop.xlsx
+++ b/Evidencias del Proyecto/Presupuesto proyecto IncluShop.xlsx
@@ -5,17 +5,20 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\benlu\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\FelipeMunhoz18-Bravo-Vargas-Munoz-Docs\Evidencias del Proyecto\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8794AB54-3F3B-412C-92F8-D81D7C369948}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E8CD408-B10E-4729-9E27-E41B8E18C78D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C9B0B423-4A3A-4590-9382-24C0D8B6837F}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{C9B0B423-4A3A-4590-9382-24C0D8B6837F}"/>
   </bookViews>
   <sheets>
     <sheet name="Contexto" sheetId="3" r:id="rId1"/>
     <sheet name="Proyecto con subscripción" sheetId="1" r:id="rId2"/>
   </sheets>
+  <externalReferences>
+    <externalReference r:id="rId3"/>
+  </externalReferences>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -35,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="45">
   <si>
     <t>Ingresos</t>
   </si>
@@ -115,9 +118,6 @@
     <t>Licencias</t>
   </si>
   <si>
-    <t>Notebooks (2)</t>
-  </si>
-  <si>
     <t>Total Compras</t>
   </si>
   <si>
@@ -167,6 +167,12 @@
   </si>
   <si>
     <t>El proyecto dura 5 meses, y a partir de mes 6 se inician las ventas, por lo cual necesitamos un vendedor que nos ayude a promocionar y vender. En este caso se asume que los primeros 5 meses son de pérdida ya que no hay ingresos y ustedes están desarrollando, esto no sería viable si tuvieran que pagar sueldos a otros programadores.</t>
+  </si>
+  <si>
+    <t>Notebooks (2) y Computadores</t>
+  </si>
+  <si>
+    <t>Gastos G/I</t>
   </si>
 </sst>
 </file>
@@ -398,7 +404,7 @@
     <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="41" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
@@ -448,9 +454,6 @@
     <xf numFmtId="41" fontId="0" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Millares [0]" xfId="1" builtinId="6"/>
@@ -468,6 +471,92 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <sheetNames>
+      <sheetName val="Plan de costos"/>
+      <sheetName val="Flujo de caja"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0">
+        <row r="4">
+          <cell r="F4">
+            <v>1670000</v>
+          </cell>
+        </row>
+        <row r="5">
+          <cell r="F5">
+            <v>1330000</v>
+          </cell>
+        </row>
+        <row r="8">
+          <cell r="F8">
+            <v>1250000</v>
+          </cell>
+        </row>
+        <row r="12">
+          <cell r="C12">
+            <v>649990</v>
+          </cell>
+        </row>
+        <row r="13">
+          <cell r="E13">
+            <v>149950</v>
+          </cell>
+        </row>
+        <row r="14">
+          <cell r="E14">
+            <v>250000</v>
+          </cell>
+        </row>
+        <row r="15">
+          <cell r="C15">
+            <v>750000</v>
+          </cell>
+        </row>
+        <row r="18">
+          <cell r="D18">
+            <v>1120000</v>
+          </cell>
+        </row>
+        <row r="19">
+          <cell r="D19">
+            <v>250000</v>
+          </cell>
+        </row>
+        <row r="20">
+          <cell r="D20">
+            <v>450000</v>
+          </cell>
+        </row>
+        <row r="21">
+          <cell r="D21">
+            <v>2000000</v>
+          </cell>
+        </row>
+        <row r="24">
+          <cell r="D24">
+            <v>100000</v>
+          </cell>
+        </row>
+        <row r="25">
+          <cell r="D25">
+            <v>175000</v>
+          </cell>
+        </row>
+        <row r="27">
+          <cell r="D27">
+            <v>100000</v>
+          </cell>
+        </row>
+      </sheetData>
+      <sheetData sheetId="1" refreshError="1"/>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -767,7 +856,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E17C452-4C71-4BC4-95A6-D021236F6BDA}">
-  <dimension ref="C3:C17"/>
+  <dimension ref="C3:C12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="118" style="19" customWidth="1"/>
@@ -775,49 +864,34 @@
   <sheetData>
     <row r="3" spans="3:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C3" s="21" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4" spans="3:3" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="3:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C5" s="20" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="6" spans="3:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="C6" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="7" spans="3:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C7" s="20" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8" spans="3:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C8" s="20" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="11" spans="3:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C11" s="21"/>
     </row>
     <row r="12" spans="3:3" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
-    <row r="13" spans="3:3" x14ac:dyDescent="0.3">
-      <c r="C13" s="29"/>
-    </row>
-    <row r="14" spans="3:3" x14ac:dyDescent="0.3">
-      <c r="C14" s="29"/>
-    </row>
-    <row r="15" spans="3:3" x14ac:dyDescent="0.3">
-      <c r="C15" s="29"/>
-    </row>
-    <row r="16" spans="3:3" x14ac:dyDescent="0.3">
-      <c r="C16" s="29"/>
-    </row>
-    <row r="17" spans="3:3" x14ac:dyDescent="0.3">
-      <c r="C17" s="29"/>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -826,7 +900,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EB435535-48A3-4C15-8A91-448AD68B5478}">
-  <dimension ref="B1:T40"/>
+  <dimension ref="B1:T41"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.33203125" customWidth="1"/>
@@ -835,13 +909,18 @@
     <col min="4" max="4" width="15.5546875" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="7" width="11.44140625" style="1"/>
     <col min="8" max="8" width="13.88671875" style="1" customWidth="1"/>
-    <col min="9" max="14" width="10" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="20" width="10" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.77734375" style="1" customWidth="1"/>
+    <col min="10" max="10" width="11" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.77734375" style="1" customWidth="1"/>
+    <col min="12" max="12" width="11" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.44140625" style="1" customWidth="1"/>
+    <col min="14" max="14" width="11" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="20" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:20" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C1" s="28" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D1" s="28"/>
       <c r="E1" s="28"/>
@@ -849,7 +928,7 @@
       <c r="G1" s="28"/>
       <c r="H1" s="28"/>
       <c r="I1" s="27" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="J1" s="27"/>
       <c r="K1" s="27"/>
@@ -857,7 +936,7 @@
       <c r="M1" s="27"/>
       <c r="N1" s="27"/>
       <c r="O1" s="23" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="P1" s="23"/>
       <c r="Q1" s="23"/>
@@ -968,51 +1047,51 @@
       </c>
       <c r="I4" s="10">
         <f t="shared" ref="I4:T4" si="0">$M$21</f>
-        <v>25000</v>
+        <v>49990</v>
       </c>
       <c r="J4" s="10">
         <f t="shared" si="0"/>
-        <v>25000</v>
+        <v>49990</v>
       </c>
       <c r="K4" s="10">
         <f t="shared" si="0"/>
-        <v>25000</v>
+        <v>49990</v>
       </c>
       <c r="L4" s="10">
         <f t="shared" si="0"/>
-        <v>25000</v>
+        <v>49990</v>
       </c>
       <c r="M4" s="10">
         <f t="shared" si="0"/>
-        <v>25000</v>
+        <v>49990</v>
       </c>
       <c r="N4" s="10">
         <f t="shared" si="0"/>
-        <v>25000</v>
+        <v>49990</v>
       </c>
       <c r="O4" s="12">
         <f t="shared" si="0"/>
-        <v>25000</v>
+        <v>49990</v>
       </c>
       <c r="P4" s="12">
         <f t="shared" si="0"/>
-        <v>25000</v>
+        <v>49990</v>
       </c>
       <c r="Q4" s="12">
         <f t="shared" si="0"/>
-        <v>25000</v>
+        <v>49990</v>
       </c>
       <c r="R4" s="12">
         <f t="shared" si="0"/>
-        <v>25000</v>
+        <v>49990</v>
       </c>
       <c r="S4" s="12">
         <f t="shared" si="0"/>
-        <v>25000</v>
+        <v>49990</v>
       </c>
       <c r="T4" s="12">
         <f t="shared" si="0"/>
-        <v>25000</v>
+        <v>49990</v>
       </c>
     </row>
     <row r="5" spans="2:20" x14ac:dyDescent="0.3">
@@ -1039,51 +1118,51 @@
       </c>
       <c r="I5" s="10">
         <f t="shared" ref="I5:T5" si="1">$M$22</f>
-        <v>200</v>
+        <v>280</v>
       </c>
       <c r="J5" s="10">
         <f t="shared" si="1"/>
-        <v>200</v>
+        <v>280</v>
       </c>
       <c r="K5" s="10">
         <f t="shared" si="1"/>
-        <v>200</v>
+        <v>280</v>
       </c>
       <c r="L5" s="10">
         <f t="shared" si="1"/>
-        <v>200</v>
+        <v>280</v>
       </c>
       <c r="M5" s="10">
         <f t="shared" si="1"/>
-        <v>200</v>
+        <v>280</v>
       </c>
       <c r="N5" s="10">
         <f t="shared" si="1"/>
-        <v>200</v>
+        <v>280</v>
       </c>
       <c r="O5" s="12">
         <f t="shared" si="1"/>
-        <v>200</v>
+        <v>280</v>
       </c>
       <c r="P5" s="12">
         <f t="shared" si="1"/>
-        <v>200</v>
+        <v>280</v>
       </c>
       <c r="Q5" s="12">
         <f t="shared" si="1"/>
-        <v>200</v>
+        <v>280</v>
       </c>
       <c r="R5" s="12">
         <f t="shared" si="1"/>
-        <v>200</v>
+        <v>280</v>
       </c>
       <c r="S5" s="12">
         <f t="shared" si="1"/>
-        <v>200</v>
+        <v>280</v>
       </c>
       <c r="T5" s="12">
         <f t="shared" si="1"/>
-        <v>200</v>
+        <v>280</v>
       </c>
     </row>
     <row r="6" spans="2:20" x14ac:dyDescent="0.3">
@@ -1116,51 +1195,51 @@
       </c>
       <c r="I6" s="10">
         <f>I4*I5</f>
-        <v>5000000</v>
+        <v>13997200</v>
       </c>
       <c r="J6" s="10">
         <f t="shared" ref="J6:N6" si="3">J4*J5</f>
-        <v>5000000</v>
+        <v>13997200</v>
       </c>
       <c r="K6" s="10">
         <f t="shared" si="3"/>
-        <v>5000000</v>
+        <v>13997200</v>
       </c>
       <c r="L6" s="10">
         <f t="shared" si="3"/>
-        <v>5000000</v>
+        <v>13997200</v>
       </c>
       <c r="M6" s="10">
         <f t="shared" si="3"/>
-        <v>5000000</v>
+        <v>13997200</v>
       </c>
       <c r="N6" s="10">
         <f t="shared" si="3"/>
-        <v>5000000</v>
+        <v>13997200</v>
       </c>
       <c r="O6" s="12">
         <f>O4*O5</f>
-        <v>5000000</v>
+        <v>13997200</v>
       </c>
       <c r="P6" s="12">
         <f t="shared" ref="P6:T6" si="4">P4*P5</f>
-        <v>5000000</v>
+        <v>13997200</v>
       </c>
       <c r="Q6" s="12">
         <f t="shared" si="4"/>
-        <v>5000000</v>
+        <v>13997200</v>
       </c>
       <c r="R6" s="12">
         <f t="shared" si="4"/>
-        <v>5000000</v>
+        <v>13997200</v>
       </c>
       <c r="S6" s="12">
         <f t="shared" si="4"/>
-        <v>5000000</v>
+        <v>13997200</v>
       </c>
       <c r="T6" s="12">
         <f t="shared" si="4"/>
-        <v>5000000</v>
+        <v>13997200</v>
       </c>
     </row>
     <row r="7" spans="2:20" x14ac:dyDescent="0.3">
@@ -1198,51 +1277,51 @@
       <c r="H8" s="9"/>
       <c r="I8" s="10">
         <f>SUM(I6:I7)</f>
-        <v>5000000</v>
+        <v>13997200</v>
       </c>
       <c r="J8" s="10">
         <f t="shared" ref="J8:N8" si="5">SUM(J6:J7)</f>
-        <v>5000000</v>
+        <v>13997200</v>
       </c>
       <c r="K8" s="10">
         <f t="shared" si="5"/>
-        <v>5000000</v>
+        <v>13997200</v>
       </c>
       <c r="L8" s="10">
         <f t="shared" si="5"/>
-        <v>5000000</v>
+        <v>13997200</v>
       </c>
       <c r="M8" s="10">
         <f t="shared" si="5"/>
-        <v>5000000</v>
+        <v>13997200</v>
       </c>
       <c r="N8" s="10">
         <f t="shared" si="5"/>
-        <v>5000000</v>
+        <v>13997200</v>
       </c>
       <c r="O8" s="12">
         <f>SUM(O6:O7)</f>
-        <v>5000000</v>
+        <v>13997200</v>
       </c>
       <c r="P8" s="12">
         <f t="shared" ref="P8:T8" si="6">SUM(P6:P7)</f>
-        <v>5000000</v>
+        <v>13997200</v>
       </c>
       <c r="Q8" s="12">
         <f t="shared" si="6"/>
-        <v>5000000</v>
+        <v>13997200</v>
       </c>
       <c r="R8" s="12">
         <f t="shared" si="6"/>
-        <v>5000000</v>
+        <v>13997200</v>
       </c>
       <c r="S8" s="12">
         <f t="shared" si="6"/>
-        <v>5000000</v>
+        <v>13997200</v>
       </c>
       <c r="T8" s="12">
         <f t="shared" si="6"/>
-        <v>5000000</v>
+        <v>13997200</v>
       </c>
     </row>
     <row r="9" spans="2:20" x14ac:dyDescent="0.3">
@@ -1314,27 +1393,27 @@
       </c>
       <c r="C12" s="9">
         <f t="shared" ref="C12:H12" si="7">$I$27</f>
-        <v>3500000</v>
+        <v>5580000</v>
       </c>
       <c r="D12" s="9">
         <f t="shared" si="7"/>
-        <v>3500000</v>
+        <v>5580000</v>
       </c>
       <c r="E12" s="9">
         <f t="shared" si="7"/>
-        <v>3500000</v>
+        <v>5580000</v>
       </c>
       <c r="F12" s="9">
         <f t="shared" si="7"/>
-        <v>3500000</v>
+        <v>5580000</v>
       </c>
       <c r="G12" s="9">
         <f t="shared" si="7"/>
-        <v>3500000</v>
+        <v>5580000</v>
       </c>
       <c r="H12" s="9">
         <f t="shared" si="7"/>
-        <v>3500000</v>
+        <v>5580000</v>
       </c>
       <c r="I12" s="10"/>
       <c r="J12" s="10"/>
@@ -1355,75 +1434,75 @@
       </c>
       <c r="C13" s="9">
         <f t="shared" ref="C13:T13" si="8">$I$33</f>
-        <v>100000</v>
+        <v>375000</v>
       </c>
       <c r="D13" s="9">
         <f t="shared" si="8"/>
-        <v>100000</v>
+        <v>375000</v>
       </c>
       <c r="E13" s="9">
         <f t="shared" si="8"/>
-        <v>100000</v>
+        <v>375000</v>
       </c>
       <c r="F13" s="9">
         <f t="shared" si="8"/>
-        <v>100000</v>
+        <v>375000</v>
       </c>
       <c r="G13" s="9">
         <f t="shared" si="8"/>
-        <v>100000</v>
+        <v>375000</v>
       </c>
       <c r="H13" s="9">
         <f t="shared" si="8"/>
-        <v>100000</v>
+        <v>375000</v>
       </c>
       <c r="I13" s="10">
         <f t="shared" si="8"/>
-        <v>100000</v>
+        <v>375000</v>
       </c>
       <c r="J13" s="10">
         <f t="shared" si="8"/>
-        <v>100000</v>
+        <v>375000</v>
       </c>
       <c r="K13" s="10">
         <f t="shared" si="8"/>
-        <v>100000</v>
+        <v>375000</v>
       </c>
       <c r="L13" s="10">
         <f t="shared" si="8"/>
-        <v>100000</v>
+        <v>375000</v>
       </c>
       <c r="M13" s="10">
         <f t="shared" si="8"/>
-        <v>100000</v>
+        <v>375000</v>
       </c>
       <c r="N13" s="10">
         <f t="shared" si="8"/>
-        <v>100000</v>
+        <v>375000</v>
       </c>
       <c r="O13" s="12">
         <f t="shared" si="8"/>
-        <v>100000</v>
+        <v>375000</v>
       </c>
       <c r="P13" s="12">
         <f t="shared" si="8"/>
-        <v>100000</v>
+        <v>375000</v>
       </c>
       <c r="Q13" s="12">
         <f t="shared" si="8"/>
-        <v>100000</v>
+        <v>375000</v>
       </c>
       <c r="R13" s="12">
         <f t="shared" si="8"/>
-        <v>100000</v>
+        <v>375000</v>
       </c>
       <c r="S13" s="12">
         <f t="shared" si="8"/>
-        <v>100000</v>
+        <v>375000</v>
       </c>
       <c r="T13" s="12">
         <f t="shared" si="8"/>
-        <v>100000</v>
+        <v>375000</v>
       </c>
     </row>
     <row r="14" spans="2:20" x14ac:dyDescent="0.3">
@@ -1490,8 +1569,8 @@
         <v>24</v>
       </c>
       <c r="C15" s="9">
-        <f>I39</f>
-        <v>1400000</v>
+        <f>I40</f>
+        <v>7969930</v>
       </c>
       <c r="D15" s="9"/>
       <c r="E15" s="9"/>
@@ -1517,75 +1596,75 @@
       </c>
       <c r="C16" s="9">
         <f>SUM(C12:C15)</f>
-        <v>5000000</v>
+        <v>13924930</v>
       </c>
       <c r="D16" s="9">
         <f t="shared" ref="D16:N16" si="10">SUM(D12:D15)</f>
-        <v>3600000</v>
+        <v>5955000</v>
       </c>
       <c r="E16" s="9">
         <f t="shared" si="10"/>
-        <v>3600000</v>
+        <v>5955000</v>
       </c>
       <c r="F16" s="9">
         <f t="shared" si="10"/>
-        <v>3600000</v>
+        <v>5955000</v>
       </c>
       <c r="G16" s="9">
         <f t="shared" si="10"/>
-        <v>3600000</v>
+        <v>5955000</v>
       </c>
       <c r="H16" s="9">
         <f t="shared" si="10"/>
-        <v>3600000</v>
+        <v>5955000</v>
       </c>
       <c r="I16" s="10">
         <f t="shared" si="10"/>
-        <v>1100000</v>
+        <v>1375000</v>
       </c>
       <c r="J16" s="10">
         <f t="shared" si="10"/>
-        <v>1100000</v>
+        <v>1375000</v>
       </c>
       <c r="K16" s="10">
         <f t="shared" si="10"/>
-        <v>1100000</v>
+        <v>1375000</v>
       </c>
       <c r="L16" s="10">
         <f t="shared" si="10"/>
-        <v>1100000</v>
+        <v>1375000</v>
       </c>
       <c r="M16" s="10">
         <f t="shared" si="10"/>
-        <v>1100000</v>
+        <v>1375000</v>
       </c>
       <c r="N16" s="10">
         <f t="shared" si="10"/>
-        <v>1100000</v>
+        <v>1375000</v>
       </c>
       <c r="O16" s="12">
         <f t="shared" ref="O16" si="11">SUM(O12:O15)</f>
-        <v>1100000</v>
+        <v>1375000</v>
       </c>
       <c r="P16" s="12">
         <f t="shared" ref="P16" si="12">SUM(P12:P15)</f>
-        <v>1100000</v>
+        <v>1375000</v>
       </c>
       <c r="Q16" s="12">
         <f t="shared" ref="Q16" si="13">SUM(Q12:Q15)</f>
-        <v>1100000</v>
+        <v>1375000</v>
       </c>
       <c r="R16" s="12">
         <f t="shared" ref="R16" si="14">SUM(R12:R15)</f>
-        <v>1100000</v>
+        <v>1375000</v>
       </c>
       <c r="S16" s="12">
         <f t="shared" ref="S16" si="15">SUM(S12:S15)</f>
-        <v>1100000</v>
+        <v>1375000</v>
       </c>
       <c r="T16" s="12">
         <f t="shared" ref="T16" si="16">SUM(T12:T15)</f>
-        <v>1100000</v>
+        <v>1375000</v>
       </c>
     </row>
     <row r="17" spans="2:20" x14ac:dyDescent="0.3">
@@ -1613,89 +1692,89 @@
         <v>5</v>
       </c>
       <c r="C18" s="9">
-        <f t="shared" ref="C18:N18" si="17">C8-C16</f>
-        <v>-5000000</v>
+        <f>C8-C16</f>
+        <v>-13924930</v>
       </c>
       <c r="D18" s="9">
-        <f t="shared" si="17"/>
-        <v>-3600000</v>
+        <f t="shared" ref="C18:N18" si="17">D8-D16</f>
+        <v>-5955000</v>
       </c>
       <c r="E18" s="9">
         <f t="shared" si="17"/>
-        <v>-3600000</v>
+        <v>-5955000</v>
       </c>
       <c r="F18" s="9">
         <f t="shared" si="17"/>
-        <v>-3600000</v>
+        <v>-5955000</v>
       </c>
       <c r="G18" s="9">
         <f t="shared" si="17"/>
-        <v>-3600000</v>
+        <v>-5955000</v>
       </c>
       <c r="H18" s="9">
         <f t="shared" si="17"/>
-        <v>-3600000</v>
+        <v>-5955000</v>
       </c>
       <c r="I18" s="10">
-        <f t="shared" si="17"/>
-        <v>3900000</v>
+        <f>I8-I16</f>
+        <v>12622200</v>
       </c>
       <c r="J18" s="10">
         <f t="shared" si="17"/>
-        <v>3900000</v>
+        <v>12622200</v>
       </c>
       <c r="K18" s="10">
         <f t="shared" si="17"/>
-        <v>3900000</v>
+        <v>12622200</v>
       </c>
       <c r="L18" s="10">
-        <f t="shared" si="17"/>
-        <v>3900000</v>
+        <f>L8-L16</f>
+        <v>12622200</v>
       </c>
       <c r="M18" s="10">
         <f t="shared" si="17"/>
-        <v>3900000</v>
+        <v>12622200</v>
       </c>
       <c r="N18" s="10">
         <f t="shared" si="17"/>
-        <v>3900000</v>
+        <v>12622200</v>
       </c>
       <c r="O18" s="12">
         <f t="shared" ref="O18:T18" si="18">O8-O16</f>
-        <v>3900000</v>
+        <v>12622200</v>
       </c>
       <c r="P18" s="12">
         <f t="shared" si="18"/>
-        <v>3900000</v>
+        <v>12622200</v>
       </c>
       <c r="Q18" s="12">
         <f t="shared" si="18"/>
-        <v>3900000</v>
+        <v>12622200</v>
       </c>
       <c r="R18" s="12">
         <f t="shared" si="18"/>
-        <v>3900000</v>
+        <v>12622200</v>
       </c>
       <c r="S18" s="12">
         <f t="shared" si="18"/>
-        <v>3900000</v>
+        <v>12622200</v>
       </c>
       <c r="T18" s="12">
         <f t="shared" si="18"/>
-        <v>3900000</v>
+        <v>12622200</v>
       </c>
     </row>
     <row r="19" spans="2:20" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="20" spans="2:20" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
       <c r="B20" s="14" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H20" s="24" t="s">
         <v>23</v>
       </c>
       <c r="I20" s="26"/>
       <c r="K20" s="24" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="L20" s="25"/>
       <c r="M20" s="26"/>
@@ -1706,13 +1785,13 @@
       </c>
       <c r="C21" s="3">
         <f>SUM(C16:H16)</f>
-        <v>23000000</v>
+        <v>43699930</v>
       </c>
       <c r="K21" s="15" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="M21" s="15">
-        <v>25000</v>
+        <v>49990</v>
       </c>
     </row>
     <row r="22" spans="2:20" x14ac:dyDescent="0.3">
@@ -1729,10 +1808,10 @@
       </c>
       <c r="I22" s="22"/>
       <c r="K22" s="15" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="M22" s="15">
-        <v>200</v>
+        <v>280</v>
       </c>
     </row>
     <row r="23" spans="2:20" x14ac:dyDescent="0.3">
@@ -1741,17 +1820,18 @@
       </c>
       <c r="C23" s="5">
         <f>NPV($C$22,C18:N18)</f>
-        <v>-6577189.509997311</v>
+        <v>1862159.037077425</v>
       </c>
       <c r="D23" s="1" t="str">
         <f>IF(C23&gt;0,"==&gt; Proyecto viable","==&gt; Proyecto no viable")</f>
-        <v>==&gt; Proyecto no viable</v>
+        <v>==&gt; Proyecto viable</v>
       </c>
       <c r="H23" s="15" t="s">
         <v>16</v>
       </c>
       <c r="I23" s="15">
-        <v>800000</v>
+        <f>'[1]Plan de costos'!$F$5</f>
+        <v>1330000</v>
       </c>
     </row>
     <row r="24" spans="2:20" x14ac:dyDescent="0.3">
@@ -1759,18 +1839,20 @@
         <v>17</v>
       </c>
       <c r="I24" s="15">
-        <v>800000</v>
+        <f>I23</f>
+        <v>1330000</v>
       </c>
     </row>
     <row r="25" spans="2:20" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B25" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="H25" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="H25" s="15" t="s">
-        <v>38</v>
-      </c>
       <c r="I25" s="15">
-        <v>1200000</v>
+        <f>'[1]Plan de costos'!$F$4</f>
+        <v>1670000</v>
       </c>
     </row>
     <row r="26" spans="2:20" ht="15" thickTop="1" x14ac:dyDescent="0.3">
@@ -1778,14 +1860,15 @@
         <v>15</v>
       </c>
       <c r="C26" s="3">
-        <f>SUM(C20:H20)</f>
-        <v>0</v>
+        <f>C21</f>
+        <v>43699930</v>
       </c>
       <c r="H26" s="15" t="s">
         <v>18</v>
       </c>
       <c r="I26" s="15">
-        <v>700000</v>
+        <f>'[1]Plan de costos'!$F$8</f>
+        <v>1250000</v>
       </c>
     </row>
     <row r="27" spans="2:20" x14ac:dyDescent="0.3">
@@ -1802,7 +1885,7 @@
       </c>
       <c r="I27" s="16">
         <f>SUM(I23:I26)</f>
-        <v>3500000</v>
+        <v>5580000</v>
       </c>
     </row>
     <row r="28" spans="2:20" x14ac:dyDescent="0.3">
@@ -1811,14 +1894,14 @@
       </c>
       <c r="C28" s="5">
         <f>NPV($C$27,C18:T18)</f>
-        <v>582466.05458529235</v>
+        <v>25034108.900481153</v>
       </c>
       <c r="D28" s="1" t="str">
         <f>IF(C28&gt;0,"==&gt; Proyecto viable","==&gt; Proyecto no viable")</f>
         <v>==&gt; Proyecto viable</v>
       </c>
       <c r="H28" s="17" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="I28" s="17">
         <v>1000000</v>
@@ -1835,7 +1918,8 @@
         <v>20</v>
       </c>
       <c r="I30" s="15">
-        <v>30000</v>
+        <f>'[1]Plan de costos'!$D$25</f>
+        <v>175000</v>
       </c>
     </row>
     <row r="31" spans="2:20" x14ac:dyDescent="0.3">
@@ -1843,7 +1927,8 @@
         <v>21</v>
       </c>
       <c r="I31" s="15">
-        <v>30000</v>
+        <f>'[1]Plan de costos'!$D$24</f>
+        <v>100000</v>
       </c>
     </row>
     <row r="32" spans="2:20" x14ac:dyDescent="0.3">
@@ -1851,16 +1936,17 @@
         <v>22</v>
       </c>
       <c r="I32" s="15">
-        <v>40000</v>
+        <f>'[1]Plan de costos'!$D$27</f>
+        <v>100000</v>
       </c>
     </row>
     <row r="33" spans="8:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="H33" s="18" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I33" s="18">
         <f>SUM(I30:I32)</f>
-        <v>100000</v>
+        <v>375000</v>
       </c>
     </row>
     <row r="34" spans="8:9" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
@@ -1872,10 +1958,11 @@
     </row>
     <row r="36" spans="8:9" x14ac:dyDescent="0.3">
       <c r="H36" s="15" t="s">
-        <v>26</v>
+        <v>43</v>
       </c>
       <c r="I36" s="15">
-        <v>1200000</v>
+        <f>2*'[1]Plan de costos'!$C$12+3*'[1]Plan de costos'!$C$15</f>
+        <v>3549980</v>
       </c>
     </row>
     <row r="37" spans="8:9" x14ac:dyDescent="0.3">
@@ -1890,18 +1977,30 @@
       <c r="H38" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="I38" s="15"/>
-    </row>
-    <row r="39" spans="8:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="H39" s="18" t="s">
-        <v>27</v>
-      </c>
-      <c r="I39" s="18">
-        <f>SUM(I36:I38)</f>
-        <v>1400000</v>
-      </c>
-    </row>
-    <row r="40" spans="8:9" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+      <c r="I38" s="15">
+        <f>SUM('[1]Plan de costos'!$E$13:$E$14)</f>
+        <v>399950</v>
+      </c>
+    </row>
+    <row r="39" spans="8:9" x14ac:dyDescent="0.3">
+      <c r="H39" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="I39" s="1">
+        <f>SUM('[1]Plan de costos'!$D$18:$D$21)</f>
+        <v>3820000</v>
+      </c>
+    </row>
+    <row r="40" spans="8:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="H40" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="I40" s="18">
+        <f>SUM(I36:I39)</f>
+        <v>7969930</v>
+      </c>
+    </row>
+    <row r="41" spans="8:9" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="H35:I35"/>

</xml_diff>